<commit_message>
Refonte v2 : exercices annuels, plafonds, nouvelle arborescence app/, nettoyage
</commit_message>
<xml_diff>
--- a/GestionArticles/documents_pdf/APP-2026-0003.xlsx
+++ b/GestionArticles/documents_pdf/APP-2026-0003.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -115,6 +115,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -482,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -518,7 +521,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
     </row>
@@ -569,12 +572,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Anti-crache nettoyant contact talk pour appareil électroniques</t>
+          <t>ADAPTATEUR HDMI /VGA</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -583,24 +586,24 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>455</v>
+        <v>442</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>910</v>
+        <v>442</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Bouteille (100 ml) de recharge couleur jaune impriment Canon Maxify GX3040</t>
+          <t>Anti-crache nettoyant contact talk pour appareil électroniques</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -609,83 +612,293 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>10400</v>
+        <v>455</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>10400</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>CABLE TELEPHONIQUE 2 PAIRES DIAMETRE 6/10 MM</t>
+          <t>Bouteille  (100 ml) de recharge couleur rouge impriment Canon Maxify GX3040</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Mètre</t>
+          <t>Unité</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>195</v>
+        <v>13650</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>195</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
+          <t>Câble HDMI /VGA</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>442</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
           <t>CABLE RESEAU FTP CAT 06</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Mètre</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D11" s="8" t="n">
         <v>13000</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>CÂBLE RÉSEAU RJ45 100 mètres</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>4095</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>4095</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>CÂBLE RÉSEAU RJ45 100 mètres</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>4095</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>4095</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>CÂBLE SATA</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>CÂBLE SATA</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="8" t="n">
-        <v>39000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="F15" s="8" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>CABLE TELEPHONIQUE 2 PAIRES DIAMETRE 6/10 MM</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>195</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>CABLE TELEPHONIQUE 2 PAIRES DIAMETRE 6/10 MM</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Mètre</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>195</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>TOTAL HT</t>
         </is>
       </c>
-      <c r="F11" s="11" t="n">
-        <v>50505</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="F18" s="11" t="n">
+        <v>36777</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>TVA 19%</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>6987.63</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL TTC</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>43764.63</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Document généré par l'application de gestion des articles.</t>
         </is>

</xml_diff>